<commit_message>
chore: sync public CommsBio release package
</commit_message>
<xml_diff>
--- a/manuscript/submission_data/source_data/Source_Data_Figure_1.xlsx
+++ b/manuscript/submission_data/source_data/Source_Data_Figure_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Panel_A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Panel_B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Panel_C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Panel_D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel_A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel_B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel_C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel_D" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70971,7 +70971,7 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
@@ -71652,7 +71652,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>passes_stage1_default_epoch_rule; mixed_or_partial_prn_epoch; passes_stage1_default_epoch_rule; informative_but_bounds_wide; prn_free_epoch</t>
+          <t>passes_stage1_default_epoch_rule; mixed_or_partial_prn_epoch; passes_stage1_default_epoch_rule; prn_free_epoch</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -71672,7 +71672,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -71687,7 +71687,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>jpn_pre2012_mixed_ap</t>
+          <t>jpn_pre2012_mixed_ap; jpn_ap_without_prn</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -71702,7 +71702,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>70</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -71712,17 +71712,17 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>12</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>0.6219512195121951</t>
+          <t>0.8536585365853658</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>0.4615384615384615</t>
+          <t>0.2333333333333333</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -71863,12 +71863,12 @@
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>jpn_pre2012_mixed_ap=23; jpn_ap_without_prn=28</t>
+          <t>jpn_pre2012_mixed_ap=23; jpn_ap_without_prn=47</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>jpn_pre2012_mixed_ap=0.233; jpn_ap_without_prn=0.462</t>
+          <t>jpn_pre2012_mixed_ap=0.233; jpn_ap_without_prn=0.096</t>
         </is>
       </c>
       <c r="AW14" t="inlineStr">
@@ -72212,22 +72212,22 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>923</t>
+          <t>908</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>534</t>
+          <t>517</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>43</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>0.9705573080967402</t>
+          <t>0.9547844374342797</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -72272,7 +72272,7 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
@@ -72377,12 +72377,12 @@
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>usa_wp_only=21; usa_transition_mixed=6; usa_ap_prn_background=896</t>
+          <t>usa_wp_only=21; usa_transition_mixed=6; usa_ap_prn_background=881</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>usa_wp_only=0.087; usa_transition_mixed=0.333; usa_ap_prn_background=0.025</t>
+          <t>usa_wp_only=0.087; usa_transition_mixed=0.333; usa_ap_prn_background=0.041</t>
         </is>
       </c>
       <c r="AW16" t="inlineStr">
@@ -72419,7 +72419,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>promoted_from_screening; passes_stage1_default_epoch_rule; promoted_from_screening; passes_stage1_default_epoch_rule; informative_but_bounds_wide</t>
+          <t>promoted_from_screening; passes_stage1_default_epoch_rule</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -72439,7 +72439,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -72454,7 +72454,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>gbr_wp_only</t>
+          <t>gbr_wp_only; gbr_ap_prn_positive</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -72469,7 +72469,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -72479,17 +72479,17 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>0.5517241379310345</t>
+          <t>0.5862068965517241</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>0.4666666666666667</t>
+          <t>0.4285714285714285</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -72626,12 +72626,12 @@
       </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>gbr_wp_only=8; gbr_ap_prn_positive=8</t>
+          <t>gbr_wp_only=8; gbr_ap_prn_positive=9</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>gbr_wp_only=0.429; gbr_ap_prn_positive=0.467</t>
+          <t>gbr_wp_only=0.429; gbr_ap_prn_positive=0.400</t>
         </is>
       </c>
       <c r="AW17" t="inlineStr">
@@ -72971,7 +72971,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>711</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -72981,17 +72981,17 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>140</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.8343125734430082</t>
+          <t>0.8354876615746181</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.1617473435655254</t>
+          <t>0.1605667060212514</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -73132,12 +73132,12 @@
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>chn_wp_only=0; chn_transition_mixed=0; chn_ap_mixed=710</t>
+          <t>chn_wp_only=0; chn_transition_mixed=0; chn_ap_mixed=711</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>chn_wp_only=1.000; chn_transition_mixed=NA; chn_ap_mixed=0.162</t>
+          <t>chn_wp_only=1.000; chn_transition_mixed=NA; chn_ap_mixed=0.161</t>
         </is>
       </c>
       <c r="AW19" t="inlineStr">
@@ -73461,7 +73461,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -73471,17 +73471,17 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>0.1111111111111111</t>
+          <t>0.8888888888888888</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.125</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -73618,12 +73618,12 @@
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>esp_wp_only=0; esp_transition_mixed=0; esp_ap_with_prn=1; esp_booster_modified_uncertain=0</t>
+          <t>esp_wp_only=0; esp_transition_mixed=0; esp_ap_with_prn=1; esp_booster_modified_uncertain=7</t>
         </is>
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>esp_wp_only=NA; esp_transition_mixed=NA; esp_ap_with_prn=0.000; esp_booster_modified_uncertain=1.000</t>
+          <t>esp_wp_only=NA; esp_transition_mixed=NA; esp_ap_with_prn=0.000; esp_booster_modified_uncertain=0.125</t>
         </is>
       </c>
       <c r="AW21" t="inlineStr">
@@ -73698,7 +73698,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -73708,17 +73708,17 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>13</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.7692307692307693</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -73855,12 +73855,12 @@
       </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>fin_wp_only=0; fin_ap_without_prn=0; fin_ap_with_prn=4</t>
+          <t>fin_wp_only=3; fin_ap_without_prn=0; fin_ap_with_prn=4</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>fin_wp_only=1.000; fin_ap_without_prn=1.000; fin_ap_with_prn=0.000</t>
+          <t>fin_wp_only=0.769; fin_ap_without_prn=1.000; fin_ap_with_prn=0.000</t>
         </is>
       </c>
       <c r="AW22" t="inlineStr">
@@ -73947,7 +73947,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -73957,17 +73957,17 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.6363636363636364</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>0.3888888888888888</t>
+          <t>0.2222222222222222</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -74108,12 +74108,12 @@
       </c>
       <c r="AU23" t="inlineStr">
         <is>
-          <t>fra_wp_only=0; fra_ap_mixed=11</t>
+          <t>fra_wp_only=0; fra_ap_mixed=14</t>
         </is>
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>fra_wp_only=1.000; fra_ap_mixed=0.389</t>
+          <t>fra_wp_only=1.000; fra_ap_mixed=0.222</t>
         </is>
       </c>
       <c r="AW23" t="inlineStr">

</xml_diff>